<commit_message>
rerun on 3 newest version
</commit_message>
<xml_diff>
--- a/2016/results_seqcardenc.xlsx
+++ b/2016/results_seqcardenc.xlsx
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="I2" t="inlineStr"/>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.32</v>
+        <v>0.38</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -870,7 +870,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.31</v>
+        <v>0.37</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.33</v>
+        <v>0.37</v>
       </c>
       <c r="I14" t="inlineStr"/>
     </row>
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="I16" t="inlineStr"/>
     </row>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="I18" t="inlineStr"/>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="I20" t="inlineStr"/>
     </row>
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="I21" t="inlineStr"/>
     </row>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>0.37</v>
+        <v>0.34</v>
       </c>
       <c r="I22" t="inlineStr"/>
     </row>
@@ -1320,7 +1320,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0.33</v>
+        <v>0.38</v>
       </c>
       <c r="I24" t="inlineStr"/>
     </row>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="I25" t="inlineStr"/>
     </row>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="I26" t="inlineStr"/>
     </row>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="I28" t="inlineStr"/>
     </row>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="I29" t="inlineStr"/>
     </row>
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0.36</v>
+        <v>0.45</v>
       </c>
       <c r="I30" t="inlineStr"/>
     </row>
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>0.33</v>
+        <v>0.37</v>
       </c>
       <c r="I32" t="inlineStr"/>
     </row>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="I33" t="inlineStr"/>
     </row>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="I34" t="inlineStr"/>
     </row>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0.33</v>
+        <v>0.38</v>
       </c>
       <c r="I35" t="inlineStr"/>
     </row>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0.32</v>
+        <v>0.36</v>
       </c>
       <c r="I36" t="inlineStr"/>
     </row>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="I37" t="inlineStr"/>
     </row>
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.35</v>
+        <v>0.39</v>
       </c>
       <c r="I2" t="inlineStr"/>
     </row>
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.34</v>
+        <v>0.44</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.43</v>
+        <v>0.37</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.33</v>
+        <v>0.38</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.4</v>
+        <v>0.46</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.4</v>
+        <v>0.43</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.35</v>
+        <v>0.42</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -2232,7 +2232,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0.39</v>
+        <v>0.43</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -2306,7 +2306,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.34</v>
+        <v>0.38</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -2343,7 +2343,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.34</v>
+        <v>0.37</v>
       </c>
       <c r="I14" t="inlineStr"/>
     </row>
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="I15" t="inlineStr"/>
     </row>
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="I16" t="inlineStr"/>
     </row>
@@ -2454,7 +2454,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.38</v>
+        <v>0.4</v>
       </c>
       <c r="I17" t="inlineStr"/>
     </row>
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="I18" t="inlineStr"/>
     </row>
@@ -2528,7 +2528,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="I19" t="inlineStr"/>
     </row>
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="I20" t="inlineStr"/>
     </row>
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="I21" t="inlineStr"/>
     </row>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>0.32</v>
+        <v>0.4</v>
       </c>
       <c r="I22" t="inlineStr"/>
     </row>
@@ -2676,7 +2676,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>0.34</v>
+        <v>0.37</v>
       </c>
       <c r="I23" t="inlineStr"/>
     </row>
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="I24" t="inlineStr"/>
     </row>
@@ -2750,7 +2750,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="I25" t="inlineStr"/>
     </row>
@@ -2824,7 +2824,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="I27" t="inlineStr"/>
     </row>
@@ -2861,7 +2861,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="I28" t="inlineStr"/>
     </row>
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0.33</v>
+        <v>0.38</v>
       </c>
       <c r="I29" t="inlineStr"/>
     </row>
@@ -2935,7 +2935,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="I30" t="inlineStr"/>
     </row>
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="I31" t="inlineStr"/>
     </row>
@@ -3046,7 +3046,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="I33" t="inlineStr"/>
     </row>
@@ -3083,7 +3083,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="I34" t="inlineStr"/>
     </row>
@@ -3120,7 +3120,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0.33</v>
+        <v>0.4</v>
       </c>
       <c r="I35" t="inlineStr"/>
     </row>
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0.32</v>
+        <v>0.38</v>
       </c>
       <c r="I36" t="inlineStr"/>
     </row>
@@ -3194,7 +3194,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="I37" t="inlineStr"/>
     </row>
@@ -3292,7 +3292,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>5.17</v>
+        <v>5.38</v>
       </c>
       <c r="I2" t="inlineStr"/>
     </row>
@@ -3329,7 +3329,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.73</v>
+        <v>0.79</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -3366,7 +3366,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.41</v>
+        <v>0.45</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>17.85</v>
+        <v>18.96</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -3440,7 +3440,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1.25</v>
+        <v>1.23</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -3477,7 +3477,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.49</v>
+        <v>0.48</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -3514,7 +3514,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1.65</v>
+        <v>1.69</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -3551,7 +3551,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.44</v>
+        <v>0.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -3588,7 +3588,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>149.66</v>
+        <v>207.81</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>4.1</v>
+        <v>4.75</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="I14" t="inlineStr"/>
     </row>
@@ -3773,7 +3773,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
       <c r="I15" t="inlineStr"/>
     </row>
@@ -3810,7 +3810,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="I16" t="inlineStr"/>
     </row>
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="I17" t="inlineStr"/>
     </row>
@@ -3884,7 +3884,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="I18" t="inlineStr"/>
     </row>
@@ -3921,7 +3921,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="I19" t="inlineStr"/>
     </row>
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="I20" t="inlineStr"/>
     </row>
@@ -3995,7 +3995,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="I21" t="inlineStr"/>
     </row>
@@ -4032,7 +4032,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="I22" t="inlineStr"/>
     </row>
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="I23" t="inlineStr"/>
     </row>
@@ -4106,7 +4106,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="I24" t="inlineStr"/>
     </row>
@@ -4143,7 +4143,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="I25" t="inlineStr"/>
     </row>
@@ -4180,7 +4180,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="I26" t="inlineStr"/>
     </row>
@@ -4254,7 +4254,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0.37</v>
+        <v>0.38</v>
       </c>
       <c r="I28" t="inlineStr"/>
     </row>
@@ -4291,7 +4291,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
       <c r="I29" t="inlineStr"/>
     </row>
@@ -4328,7 +4328,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="I30" t="inlineStr"/>
     </row>
@@ -4365,7 +4365,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
       <c r="I31" t="inlineStr"/>
     </row>
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>0.39</v>
+        <v>0.41</v>
       </c>
       <c r="I32" t="inlineStr"/>
     </row>
@@ -4476,7 +4476,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
       <c r="I34" t="inlineStr"/>
     </row>
@@ -4513,7 +4513,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0.52</v>
+        <v>0.47</v>
       </c>
       <c r="I35" t="inlineStr"/>
     </row>
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>0.41</v>
+        <v>0.43</v>
       </c>
       <c r="I37" t="inlineStr"/>
     </row>
@@ -4722,7 +4722,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -4792,11 +4792,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>FINISHED</t>
+          <t>TIMEOUT</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>231.99</v>
+        <v>300</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -4833,7 +4833,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -4870,7 +4870,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1.11</v>
+        <v>1.13</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -4944,7 +4944,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -4981,7 +4981,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.52</v>
+        <v>0.55</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -5055,7 +5055,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.22</v>
+        <v>1.31</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -5092,7 +5092,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -5129,7 +5129,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="I14" t="inlineStr"/>
     </row>
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>2.17</v>
+        <v>2.21</v>
       </c>
       <c r="I15" t="inlineStr"/>
     </row>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.93</v>
+        <v>1</v>
       </c>
       <c r="I16" t="inlineStr"/>
     </row>
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.52</v>
+        <v>0.58</v>
       </c>
       <c r="I17" t="inlineStr"/>
     </row>
@@ -5277,7 +5277,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>13.63</v>
+        <v>10.54</v>
       </c>
       <c r="I18" t="inlineStr"/>
     </row>
@@ -5314,7 +5314,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
       <c r="I19" t="inlineStr"/>
     </row>
@@ -5388,7 +5388,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0.43</v>
+        <v>0.48</v>
       </c>
       <c r="I21" t="inlineStr"/>
     </row>
@@ -5425,7 +5425,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>0.43</v>
+        <v>0.47</v>
       </c>
       <c r="I22" t="inlineStr"/>
     </row>
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>0.37</v>
+        <v>0.42</v>
       </c>
       <c r="I23" t="inlineStr"/>
     </row>
@@ -5499,7 +5499,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0.43</v>
+        <v>0.47</v>
       </c>
       <c r="I24" t="inlineStr"/>
     </row>
@@ -5536,7 +5536,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.41</v>
+        <v>0.43</v>
       </c>
       <c r="I25" t="inlineStr"/>
     </row>
@@ -5573,7 +5573,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="I26" t="inlineStr"/>
     </row>
@@ -5610,7 +5610,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>0.44</v>
+        <v>0.47</v>
       </c>
       <c r="I27" t="inlineStr"/>
     </row>
@@ -5721,7 +5721,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="I30" t="inlineStr"/>
     </row>
@@ -5758,7 +5758,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="I31" t="inlineStr"/>
     </row>
@@ -5832,7 +5832,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="I33" t="inlineStr"/>
     </row>
@@ -5869,7 +5869,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="I34" t="inlineStr"/>
     </row>
@@ -5906,7 +5906,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="I35" t="inlineStr"/>
     </row>
@@ -5943,7 +5943,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="I36" t="inlineStr"/>
     </row>
@@ -6152,7 +6152,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>9.93</v>
+        <v>11.28</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -6226,7 +6226,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>21.72</v>
+        <v>22.23</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
@@ -6263,7 +6263,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>4.35</v>
+        <v>4.39</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -6337,7 +6337,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.46</v>
+        <v>0.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -6374,7 +6374,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2.73</v>
+        <v>2.79</v>
       </c>
       <c r="I10" t="inlineStr"/>
     </row>
@@ -6411,7 +6411,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>6.96</v>
+        <v>9.43</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -6448,7 +6448,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>15.38</v>
+        <v>22.9</v>
       </c>
       <c r="I12" t="inlineStr"/>
     </row>
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -6596,7 +6596,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>2.59</v>
+        <v>2.63</v>
       </c>
       <c r="I16" t="inlineStr"/>
     </row>
@@ -6707,7 +6707,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1.83</v>
+        <v>1.89</v>
       </c>
       <c r="I19" t="inlineStr"/>
     </row>
@@ -6744,7 +6744,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.41</v>
+        <v>0.45</v>
       </c>
       <c r="I20" t="inlineStr"/>
     </row>
@@ -6781,7 +6781,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="I21" t="inlineStr"/>
     </row>
@@ -6818,7 +6818,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>0.41</v>
+        <v>0.45</v>
       </c>
       <c r="I22" t="inlineStr"/>
     </row>
@@ -6855,7 +6855,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="I23" t="inlineStr"/>
     </row>
@@ -6892,7 +6892,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0.42</v>
+        <v>0.47</v>
       </c>
       <c r="I24" t="inlineStr"/>
     </row>
@@ -6929,7 +6929,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.45</v>
+        <v>0.49</v>
       </c>
       <c r="I25" t="inlineStr"/>
     </row>
@@ -6966,7 +6966,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0.45</v>
+        <v>0.49</v>
       </c>
       <c r="I26" t="inlineStr"/>
     </row>
@@ -7003,7 +7003,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>0.49</v>
+        <v>0.54</v>
       </c>
       <c r="I27" t="inlineStr"/>
     </row>
@@ -7040,7 +7040,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0.45</v>
+        <v>0.51</v>
       </c>
       <c r="I28" t="inlineStr"/>
     </row>
@@ -7077,7 +7077,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="I29" t="inlineStr"/>
     </row>
@@ -7114,7 +7114,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.02</v>
+        <v>1.06</v>
       </c>
       <c r="I30" t="inlineStr"/>
     </row>
@@ -7151,7 +7151,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="I31" t="inlineStr"/>
     </row>
@@ -7188,7 +7188,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>0.49</v>
+        <v>0.53</v>
       </c>
       <c r="I32" t="inlineStr"/>
     </row>
@@ -7225,7 +7225,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>0.44</v>
+        <v>0.5</v>
       </c>
       <c r="I33" t="inlineStr"/>
     </row>
@@ -7262,7 +7262,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>0.43</v>
+        <v>0.47</v>
       </c>
       <c r="I34" t="inlineStr"/>
     </row>
@@ -7299,7 +7299,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0.48</v>
+        <v>0.54</v>
       </c>
       <c r="I35" t="inlineStr"/>
     </row>
@@ -7336,7 +7336,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0.61</v>
+        <v>0.65</v>
       </c>
       <c r="I36" t="inlineStr"/>
     </row>
@@ -7373,7 +7373,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>0.48</v>
+        <v>0.52</v>
       </c>
       <c r="I37" t="inlineStr"/>
     </row>

</xml_diff>